<commit_message>
Registro de desperdicios para clase remota
- python probar.py --desperdicio <modulo> "tipo" <min> "qué pasó"
- Esperas, retrabajo, cambios de tarea frenados por el WIP y trabajo a medias se registran solos
- --metricas genera registro/desperdicios_<modulo>.txt para pegar en la bitácora
- README y bitácora sin observadores
</commit_message>
<xml_diff>
--- a/Plantilla_Lean_CafeTec.xlsx
+++ b/Plantilla_Lean_CafeTec.xlsx
@@ -155,7 +155,7 @@
     <t xml:space="preserve">DURANTE</t>
   </si>
   <si>
-    <t xml:space="preserve">Los observadores anotan desperdicios en la hoja Desperdicios (equipo, tipo, minutos).</t>
+    <t xml:space="preserve">El encargado de flujo anota desperdicios con python probar.py --desperdicio. Esperas, retrabajo y cambios de tarea se registran solos.</t>
   </si>
   <si>
     <t xml:space="preserve">Detenidos esperando a alguien o algo</t>
@@ -173,7 +173,7 @@
     <t xml:space="preserve">AL FINAL</t>
   </si>
   <si>
-    <t xml:space="preserve">python probar.py --metricas &lt;modulo&gt; y pegar el .txt en la hoja Flujo, en la fila de su equipo (celda marcada ◀).</t>
+    <t xml:space="preserve">python probar.py --metricas &lt;modulo&gt;: pegar metricas_&lt;modulo&gt;.txt en Flujo (celda ◀) y desperdicios_&lt;modulo&gt;.txt en Desperdicios.</t>
   </si>
   <si>
     <t xml:space="preserve">Corregir lo que ya estaba "terminado"</t>
@@ -401,7 +401,7 @@
     <t xml:space="preserve">Registro de desperdicios</t>
   </si>
   <si>
-    <t xml:space="preserve">Lo llenan observadores, encargados de flujo y revisores en el momento en que pasa</t>
+    <t xml:space="preserve">Cada equipo pega aquí registro/desperdicios_&lt;modulo&gt;.txt en la primera fila libre (columna Día) y escribe la contramedida</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -1332,11 +1332,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="93264320"/>
-        <c:axId val="98988421"/>
+        <c:axId val="23154466"/>
+        <c:axId val="97423763"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="93264320"/>
+        <c:axId val="23154466"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1368,7 +1368,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98988421"/>
+        <c:crossAx val="97423763"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1376,7 +1376,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98988421"/>
+        <c:axId val="97423763"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1418,7 +1418,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93264320"/>
+        <c:crossAx val="23154466"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1715,11 +1715,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="43890501"/>
-        <c:axId val="64435630"/>
+        <c:axId val="32021108"/>
+        <c:axId val="18980118"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="43890501"/>
+        <c:axId val="32021108"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1751,7 +1751,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64435630"/>
+        <c:crossAx val="18980118"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1759,7 +1759,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64435630"/>
+        <c:axId val="18980118"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1801,7 +1801,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43890501"/>
+        <c:crossAx val="32021108"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3794,7 +3794,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H44" type="list">
-      <formula1>"Mismo equipo,Observador,Revisor,Profesor"</formula1>
+      <formula1>"Mismo equipo,probar.py,Revisor,Profesor"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Una sola sesión: los 6 equipos programan y el equipo organizador revisa
- probar.py: sin días; el tablero compara equipos y actividad 1 contra 3
- Bitácora: developer en Portada, revisión por el organizador, resultados por actividad
- README, REVISION.md, plantilla de PR y docstrings sin día 1/día 2
</commit_message>
<xml_diff>
--- a/Plantilla_Lean_CafeTec.xlsx
+++ b/Plantilla_Lean_CafeTec.xlsx
@@ -128,13 +128,35 @@
 </comments>
 </file>
 
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="L11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">En la fila Grupo, la espera de revisión es el promedio por PR.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="140">
   <si>
     <t xml:space="preserve">CafeTec · Bitácora Lean</t>
   </si>
   <si>
-    <t xml:space="preserve">Lean Software Development · métricas de flujo del grupo</t>
+    <t xml:space="preserve">Lean Software Development · los 6 equipos programan en la misma sesión; el equipo organizador revisa</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo se llena</t>
@@ -146,7 +168,7 @@
     <t xml:space="preserve">ANTES</t>
   </si>
   <si>
-    <t xml:space="preserve">Cada equipo escribe sus integrantes en la tabla de abajo.</t>
+    <t xml:space="preserve">Cada equipo escribe su developer e integrantes en la tabla de abajo.</t>
   </si>
   <si>
     <t xml:space="preserve">Espera</t>
@@ -164,7 +186,7 @@
     <t xml:space="preserve">AL CERRAR EL PR</t>
   </si>
   <si>
-    <t xml:space="preserve">El equipo revisor anota horas y cambios pedidos en la hoja Revisiones.</t>
+    <t xml:space="preserve">El equipo organizador revisa el PR y anota horas y cambios pedidos en la hoja Revisiones.</t>
   </si>
   <si>
     <t xml:space="preserve">Retrabajo / defecto</t>
@@ -203,7 +225,7 @@
     <t xml:space="preserve">Módulo</t>
   </si>
   <si>
-    <t xml:space="preserve">Día</t>
+    <t xml:space="preserve">Developer</t>
   </si>
   <si>
     <t xml:space="preserve">Integrantes</t>
@@ -221,48 +243,51 @@
     <t xml:space="preserve">Usuarios</t>
   </si>
   <si>
+    <t xml:space="preserve">Organizador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Funcionalidad extra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipo 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catálogo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programar lo que no se pidió</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipo 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transferencia / traspaso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipo 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Información perdida entre personas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipo 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inventario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demoras de proceso</t>
+  </si>
+  <si>
     <t xml:space="preserve">Equipo 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Funcionalidad extra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipo 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catálogo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipo 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programar lo que no se pidió</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipo 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pedidos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipo 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transferencia / traspaso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Información perdida entre personas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inventario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demoras de proceso</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reportes</t>
   </si>
   <si>
@@ -299,6 +324,9 @@
     <t xml:space="preserve">Pega aquí la salida de python probar.py --metricas &lt;modulo&gt;, empezando en la celda ◀ de tu equipo (columna Act.)</t>
   </si>
   <si>
+    <t xml:space="preserve">Revisa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Act.</t>
   </si>
   <si>
@@ -401,7 +429,7 @@
     <t xml:space="preserve">Registro de desperdicios</t>
   </si>
   <si>
-    <t xml:space="preserve">Cada equipo pega aquí registro/desperdicios_&lt;modulo&gt;.txt en la primera fila libre (columna Día) y escribe la contramedida</t>
+    <t xml:space="preserve">Cada equipo pega aquí registro/desperdicios_&lt;modulo&gt;.txt en la primera fila libre (columna Act.) y escribe la contramedida</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -428,13 +456,13 @@
     <t xml:space="preserve">Revisión de Pull Requests</t>
   </si>
   <si>
-    <t xml:space="preserve">Un renglón por equipo. Lo llena el equipo revisor al aprobar el PR (formato de hora 10:42)</t>
+    <t xml:space="preserve">El equipo organizador revisa los 6 PR. Un renglón por equipo; se llena al aprobar (formato de hora 10:42)</t>
   </si>
   <si>
     <t xml:space="preserve">Equipo autor</t>
   </si>
   <si>
-    <t xml:space="preserve">Revisor</t>
+    <t xml:space="preserve">Revisó (nombre)</t>
   </si>
   <si>
     <t xml:space="preserve">PR #</t>
@@ -455,13 +483,13 @@
     <t xml:space="preserve">Qué pidieron corregir</t>
   </si>
   <si>
-    <t xml:space="preserve">Cada cambio pedido cuenta como un defecto encontrado en revisión.</t>
+    <t xml:space="preserve">Cada cambio pedido cuenta como un defecto encontrado en revisión. Si muchos PR esperan al mismo tiempo, esa cola es desperdicio: repártanse la revisión.</t>
   </si>
   <si>
     <t xml:space="preserve">Retrospectiva y mejora continua</t>
   </si>
   <si>
-    <t xml:space="preserve">Respondan con datos de Flujo, Desperdicios y Revisiones. La mejora del día 1 la aplican los equipos del día 2</t>
+    <t xml:space="preserve">Respondan con datos de Flujo, Desperdicios, Revisiones y Resultados</t>
   </si>
   <si>
     <t xml:space="preserve">¿Qué funcionó bien?</t>
@@ -473,16 +501,13 @@
     <t xml:space="preserve">Mejora que proponemos</t>
   </si>
   <si>
-    <t xml:space="preserve">¿Se aplicó el día 2?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resultado observado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acuerdo del grupo al cerrar el día 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conclusión final: ¿la mejora redujo el lead time, la espera o los defectos? (usen la hoja Resultados)</t>
+    <t xml:space="preserve">¿La actividad 3 salió mejor que la 1? (lead y defectos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mejora que el grupo propone para la próxima vez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conclusión: ¿qué nos dicen los datos? (equipos, actividad 1 contra 3, desperdicio y espera de revisión)</t>
   </si>
   <si>
     <t xml:space="preserve">Resultados del grupo</t>
@@ -518,10 +543,13 @@
     <t xml:space="preserve">Espera revisión (min)</t>
   </si>
   <si>
-    <t xml:space="preserve">Día 1 contra día 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lead prom. por actividad</t>
+    <t xml:space="preserve">Grupo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actividad 1 contra actividad 3 (curva de aprendizaje)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actividad</t>
   </si>
   <si>
     <t xml:space="preserve">Defectos por actividad</t>
@@ -530,7 +558,7 @@
     <t xml:space="preserve">% bien a la 1a</t>
   </si>
   <si>
-    <t xml:space="preserve">Espera revisión prom.</t>
+    <t xml:space="preserve">Si la actividad 3 tiene menor lead promedio y menos defectos que la 1, el grupo aprendió durante la sesión (amplificar el aprendizaje).</t>
   </si>
   <si>
     <t xml:space="preserve">Minutos de desperdicio por tipo</t>
@@ -539,10 +567,10 @@
     <t xml:space="preserve">Tipo</t>
   </si>
   <si>
-    <t xml:space="preserve">Día 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Día 2</t>
+    <t xml:space="preserve">Minutos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registros</t>
   </si>
 </sst>
 </file>
@@ -833,7 +861,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1050,24 +1078,28 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1230,7 +1262,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Resultados!E4</c:f>
+              <c:f>Resultados!D4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1304,7 +1336,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resultados!$E$5:$E$10</c:f>
+              <c:f>Resultados!$D$5:$D$10</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1332,11 +1364,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="23154466"/>
-        <c:axId val="97423763"/>
+        <c:axId val="39444791"/>
+        <c:axId val="58556721"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="23154466"/>
+        <c:axId val="39444791"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1368,7 +1400,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97423763"/>
+        <c:crossAx val="58556721"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1376,7 +1408,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97423763"/>
+        <c:axId val="58556721"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1418,7 +1450,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23154466"/>
+        <c:crossAx val="39444791"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1496,11 +1528,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Resultados!D20</c:f>
+              <c:f>Resultados!D21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Día 1</c:v>
+                  <c:v>Minutos</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1544,7 +1576,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Resultados!$A$21:$A$27</c:f>
+              <c:f>Resultados!$A$22:$A$28</c:f>
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
@@ -1573,118 +1605,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Resultados!$D$21:$D$27</c:f>
-              <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Resultados!E20</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Día 2</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="7a2e1c"/>
-            </a:solidFill>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="7a2e1c"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:txPr>
-              <a:bodyPr wrap="none"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-              </a:p>
-            </c:txPr>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:separator> </c:separator>
-            <c:showLeaderLines val="1"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>Resultados!$A$21:$A$27</c:f>
-              <c:strCache>
-                <c:ptCount val="7"/>
-                <c:pt idx="0">
-                  <c:v>Espera</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Retrabajo / defecto</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Trabajo parcialmente hecho</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Cambio de tarea</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Funcionalidad extra</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Transferencia / traspaso</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Demoras de proceso</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Resultados!$E$21:$E$27</c:f>
+              <c:f>Resultados!$D$22:$D$28</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1715,11 +1636,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="32021108"/>
-        <c:axId val="18980118"/>
+        <c:axId val="86591652"/>
+        <c:axId val="1912190"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="32021108"/>
+        <c:axId val="86591652"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1751,7 +1672,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18980118"/>
+        <c:crossAx val="1912190"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1759,7 +1680,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18980118"/>
+        <c:axId val="1912190"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1801,7 +1722,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32021108"/>
+        <c:crossAx val="86591652"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1812,30 +1733,6 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:defRPr>
-          </a:pPr>
-        </a:p>
-      </c:txPr>
-    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
@@ -1859,14 +1756,14 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>175680</xdr:rowOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>387720</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>90000</xdr:rowOff>
+      <xdr:colOff>246600</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>90360</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1874,7 +1771,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="4370040" y="4352760"/>
+        <a:off x="4651920" y="4543560"/>
         <a:ext cx="5039640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1889,13 +1786,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>161280</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>669600</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:colOff>387720</xdr:colOff>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>14040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -1904,7 +1801,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="6562800"/>
+        <a:off x="0" y="6753240"/>
         <a:ext cx="5039640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2105,7 +2002,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="3"/>
@@ -2254,9 +2151,7 @@
       <c r="C13" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="12" t="s">
         <v>30</v>
@@ -2272,33 +2167,29 @@
       <c r="C14" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H14" s="9" t="s">
         <v>34</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="D15" s="13"/>
       <c r="E15" s="13"/>
       <c r="F15" s="12" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2306,32 +2197,28 @@
         <v>38</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>2</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="12" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="11" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="12" t="n">
-        <v>2</v>
-      </c>
+      <c r="D17" s="13"/>
       <c r="E17" s="13"/>
       <c r="F17" s="12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>43</v>
@@ -2339,30 +2226,28 @@
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="11" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>2</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
@@ -2372,26 +2257,26 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -2425,7 +2310,8 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="6" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
@@ -2436,7 +2322,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2456,7 +2342,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2482,46 +2368,46 @@
         <v>23</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="N4" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="O4" s="19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2531,14 +2417,14 @@
       <c r="B5" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="12" t="n">
-        <v>1</v>
+      <c r="C5" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F5" s="22"/>
       <c r="G5" s="22"/>
@@ -2568,14 +2454,14 @@
       <c r="B6" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="12" t="n">
-        <v>1</v>
+      <c r="C6" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="D6" s="20" t="n">
         <v>2</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F6" s="22"/>
       <c r="G6" s="22"/>
@@ -2605,14 +2491,14 @@
       <c r="B7" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="28" t="n">
-        <v>1</v>
+      <c r="C7" s="28" t="s">
+        <v>30</v>
       </c>
       <c r="D7" s="29" t="n">
         <v>3</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F7" s="31"/>
       <c r="G7" s="31"/>
@@ -2642,14 +2528,14 @@
       <c r="B8" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="37" t="n">
-        <v>1</v>
+      <c r="C8" s="37" t="s">
+        <v>30</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F8" s="39"/>
       <c r="G8" s="39"/>
@@ -2679,14 +2565,14 @@
       <c r="B9" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="37" t="n">
-        <v>1</v>
+      <c r="C9" s="37" t="s">
+        <v>30</v>
       </c>
       <c r="D9" s="38" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F9" s="39"/>
       <c r="G9" s="39"/>
@@ -2716,14 +2602,14 @@
       <c r="B10" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="43" t="n">
-        <v>1</v>
+      <c r="C10" s="43" t="s">
+        <v>30</v>
       </c>
       <c r="D10" s="44" t="n">
         <v>3</v>
       </c>
       <c r="E10" s="45" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F10" s="46"/>
       <c r="G10" s="46"/>
@@ -2748,19 +2634,19 @@
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="12" t="n">
-        <v>1</v>
+      <c r="C11" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F11" s="22"/>
       <c r="G11" s="22"/>
@@ -2785,19 +2671,19 @@
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>1</v>
+      <c r="C12" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="D12" s="20" t="n">
         <v>2</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F12" s="22"/>
       <c r="G12" s="22"/>
@@ -2822,19 +2708,19 @@
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="28" t="n">
-        <v>1</v>
+      <c r="C13" s="28" t="s">
+        <v>30</v>
       </c>
       <c r="D13" s="29" t="n">
         <v>3</v>
       </c>
       <c r="E13" s="30" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F13" s="31"/>
       <c r="G13" s="31"/>
@@ -2862,16 +2748,16 @@
         <v>38</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="37" t="n">
-        <v>2</v>
+        <v>39</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>30</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F14" s="39"/>
       <c r="G14" s="39"/>
@@ -2899,16 +2785,16 @@
         <v>38</v>
       </c>
       <c r="B15" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="37" t="n">
-        <v>2</v>
+        <v>39</v>
+      </c>
+      <c r="C15" s="37" t="s">
+        <v>30</v>
       </c>
       <c r="D15" s="38" t="n">
         <v>2</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F15" s="39"/>
       <c r="G15" s="39"/>
@@ -2936,16 +2822,16 @@
         <v>38</v>
       </c>
       <c r="B16" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="43" t="n">
-        <v>2</v>
+        <v>39</v>
+      </c>
+      <c r="C16" s="43" t="s">
+        <v>30</v>
       </c>
       <c r="D16" s="44" t="n">
         <v>3</v>
       </c>
       <c r="E16" s="45" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F16" s="46"/>
       <c r="G16" s="46"/>
@@ -2970,19 +2856,19 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="12" t="n">
-        <v>2</v>
+      <c r="C17" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F17" s="22"/>
       <c r="G17" s="22"/>
@@ -3007,19 +2893,19 @@
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="26" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B18" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="12" t="n">
-        <v>2</v>
+      <c r="C18" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="D18" s="20" t="n">
         <v>2</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F18" s="22"/>
       <c r="G18" s="22"/>
@@ -3044,19 +2930,19 @@
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="27" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B19" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="28" t="n">
-        <v>2</v>
+      <c r="C19" s="28" t="s">
+        <v>30</v>
       </c>
       <c r="D19" s="29" t="n">
         <v>3</v>
       </c>
       <c r="E19" s="30" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F19" s="31"/>
       <c r="G19" s="31"/>
@@ -3081,19 +2967,19 @@
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="37" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="37" t="n">
-        <v>2</v>
-      </c>
       <c r="D20" s="38" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F20" s="39"/>
       <c r="G20" s="39"/>
@@ -3118,19 +3004,19 @@
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="37" t="s">
         <v>30</v>
-      </c>
-      <c r="B21" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="37" t="n">
-        <v>2</v>
       </c>
       <c r="D21" s="38" t="n">
         <v>2</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F21" s="39"/>
       <c r="G21" s="39"/>
@@ -3155,19 +3041,19 @@
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="43" t="s">
         <v>30</v>
-      </c>
-      <c r="B22" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="43" t="n">
-        <v>2</v>
       </c>
       <c r="D22" s="44" t="n">
         <v>3</v>
       </c>
       <c r="E22" s="45" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F22" s="46"/>
       <c r="G22" s="46"/>
@@ -3192,7 +3078,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -3242,7 +3128,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3254,7 +3140,7 @@
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3266,28 +3152,28 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3772,7 +3658,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E46" s="48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F46" s="49" t="n">
         <f aca="false">SUM(F5:F44)</f>
@@ -3782,7 +3668,7 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B44" type="list">
-      <formula1>"1,2"</formula1>
+      <formula1>"1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C44" type="list">
@@ -3814,23 +3700,22 @@
     <tabColor rgb="FFE8A33D"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3840,11 +3725,10 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3854,38 +3738,34 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>24</v>
+        <v>103</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3895,21 +3775,16 @@
       <c r="B5" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="50"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="39"/>
       <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="51" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F5),ISNUMBER(G5)),ROUND((G5-F5)*1440,0),"")</f>
-        <v/>
-      </c>
-      <c r="I5" s="50"/>
-      <c r="J5" s="13"/>
+      <c r="G5" s="51" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E5),ISNUMBER(F5)),ROUND((F5-E5)*1440,0),"")</f>
+        <v/>
+      </c>
+      <c r="H5" s="50"/>
+      <c r="I5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
@@ -3918,117 +3793,92 @@
       <c r="B6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="50"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="39"/>
       <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="51" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F6),ISNUMBER(G6)),ROUND((G6-F6)*1440,0),"")</f>
-        <v/>
-      </c>
-      <c r="I6" s="50"/>
-      <c r="J6" s="13"/>
+      <c r="G6" s="51" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E6),ISNUMBER(F6)),ROUND((F6-E6)*1440,0),"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="50"/>
+      <c r="I6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="50"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="39"/>
       <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="51" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F7),ISNUMBER(G7)),ROUND((G7-F7)*1440,0),"")</f>
-        <v/>
-      </c>
-      <c r="I7" s="50"/>
-      <c r="J7" s="13"/>
+      <c r="G7" s="51" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E7),ISNUMBER(F7)),ROUND((F7-E7)*1440,0),"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="50"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
         <v>38</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" s="50"/>
+        <v>39</v>
+      </c>
+      <c r="C8" s="13"/>
+      <c r="D8" s="50"/>
+      <c r="E8" s="39"/>
       <c r="F8" s="39"/>
-      <c r="G8" s="39"/>
-      <c r="H8" s="51" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F8),ISNUMBER(G8)),ROUND((G8-F8)*1440,0),"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="50"/>
-      <c r="J8" s="13"/>
+      <c r="G8" s="51" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E8),ISNUMBER(F8)),ROUND((F8-E8)*1440,0),"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="50"/>
+      <c r="I8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="50"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="39"/>
       <c r="F9" s="39"/>
-      <c r="G9" s="39"/>
-      <c r="H9" s="51" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F9),ISNUMBER(G9)),ROUND((G9-F9)*1440,0),"")</f>
-        <v/>
-      </c>
-      <c r="I9" s="50"/>
-      <c r="J9" s="13"/>
+      <c r="G9" s="51" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E9),ISNUMBER(F9)),ROUND((F9-E9)*1440,0),"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="50"/>
+      <c r="I9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="50"/>
+        <v>45</v>
+      </c>
+      <c r="C10" s="13"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="39"/>
       <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="51" t="str">
-        <f aca="false">IF(AND(ISNUMBER(F10),ISNUMBER(G10)),ROUND((G10-F10)*1440,0),"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="50"/>
-      <c r="J10" s="13"/>
+      <c r="G10" s="51" t="str">
+        <f aca="false">IF(AND(ISNUMBER(E10),ISNUMBER(F10)),ROUND((F10-E10)*1440,0),"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="50"/>
+      <c r="I10" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -4048,142 +3898,106 @@
     <tabColor rgb="FFE8A33D"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>24</v>
+        <v>113</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="B5" s="13"/>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="B6" s="13"/>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>1</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
-      <c r="F7" s="38"/>
-      <c r="G7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="12" t="n">
-        <v>2</v>
-      </c>
+      <c r="B8" s="13"/>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>2</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>2</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="B10" s="13"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="52" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4192,8 +4006,6 @@
       <c r="C13" s="53"/>
       <c r="D13" s="53"/>
       <c r="E13" s="53"/>
-      <c r="F13" s="53"/>
-      <c r="G13" s="53"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="53"/>
@@ -4201,8 +4013,6 @@
       <c r="C14" s="53"/>
       <c r="D14" s="53"/>
       <c r="E14" s="53"/>
-      <c r="F14" s="53"/>
-      <c r="G14" s="53"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="53"/>
@@ -4210,12 +4020,10 @@
       <c r="C15" s="53"/>
       <c r="D15" s="53"/>
       <c r="E15" s="53"/>
-      <c r="F15" s="53"/>
-      <c r="G15" s="53"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="52" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4224,8 +4032,6 @@
       <c r="C18" s="53"/>
       <c r="D18" s="53"/>
       <c r="E18" s="53"/>
-      <c r="F18" s="53"/>
-      <c r="G18" s="53"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="53"/>
@@ -4233,8 +4039,6 @@
       <c r="C19" s="53"/>
       <c r="D19" s="53"/>
       <c r="E19" s="53"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="53"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="53"/>
@@ -4242,8 +4046,6 @@
       <c r="C20" s="53"/>
       <c r="D20" s="53"/>
       <c r="E20" s="53"/>
-      <c r="F20" s="53"/>
-      <c r="G20" s="53"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="53"/>
@@ -4251,20 +4053,12 @@
       <c r="C21" s="53"/>
       <c r="D21" s="53"/>
       <c r="E21" s="53"/>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:G15"/>
-    <mergeCell ref="A18:G21"/>
+    <mergeCell ref="A13:E15"/>
+    <mergeCell ref="A18:E21"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F10" type="list">
-      <formula1>"Sí,No,Parcial"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4281,21 +4075,20 @@
     <tabColor rgb="FF7A2E1C"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="8" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4308,11 +4101,10 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4325,7 +4117,6 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
@@ -4335,37 +4126,34 @@
         <v>23</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>24</v>
+        <v>121</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>122</v>
+        <v>63</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>61</v>
+        <v>124</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="M4" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4375,47 +4163,44 @@
       <c r="B5" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="51" t="n">
+      <c r="C5" s="51" t="n">
         <f aca="false">COUNTIFS(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$H$5:$H$22,"&gt;=0")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="D5" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$H$5:$H$22)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="24" t="str">
-        <f aca="false">IF(D5&gt;0,E5/D5,"")</f>
-        <v/>
-      </c>
-      <c r="G5" s="24" t="n">
+      <c r="E5" s="24" t="str">
+        <f aca="false">IF(C5&gt;0,D5/C5,"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$I$5:$I$22)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="25" t="str">
-        <f aca="false">IF(E5&gt;0,(E5-G5)/E5,"")</f>
-        <v/>
+      <c r="G5" s="25" t="str">
+        <f aca="false">IF(D5&gt;0,(D5-F5)/D5,"")</f>
+        <v/>
+      </c>
+      <c r="H5" s="51" t="n">
+        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$K$5:$K$22)</f>
+        <v>0</v>
       </c>
       <c r="I5" s="51" t="n">
-        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$K$5:$K$22)</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 1",Revisiones!$I$5:$I$10)</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="25" t="str">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 1",Revisiones!$H$5:$H$10)</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="25" t="str">
         <f aca="false">IF(COUNTIFS(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$A$5:$A$22,"Equipo 1",Flujo!$M$5:$M$22,"?*"))</f>
         <v/>
       </c>
-      <c r="L5" s="24" t="n">
+      <c r="K5" s="24" t="n">
         <f aca="false">SUMIF(Desperdicios!$C$5:$C$44,"Equipo 1",Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="M5" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 1",Revisiones!$H$5:$H$10)</f>
+      <c r="L5" s="51" t="n">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 1",Revisiones!$G$5:$G$10)</f>
         <v>0</v>
       </c>
     </row>
@@ -4426,98 +4211,92 @@
       <c r="B6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="51" t="n">
+      <c r="C6" s="51" t="n">
         <f aca="false">COUNTIFS(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$H$5:$H$22,"&gt;=0")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="D6" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$H$5:$H$22)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="24" t="str">
-        <f aca="false">IF(D6&gt;0,E6/D6,"")</f>
-        <v/>
-      </c>
-      <c r="G6" s="24" t="n">
+      <c r="E6" s="24" t="str">
+        <f aca="false">IF(C6&gt;0,D6/C6,"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$I$5:$I$22)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="25" t="str">
-        <f aca="false">IF(E6&gt;0,(E6-G6)/E6,"")</f>
-        <v/>
+      <c r="G6" s="25" t="str">
+        <f aca="false">IF(D6&gt;0,(D6-F6)/D6,"")</f>
+        <v/>
+      </c>
+      <c r="H6" s="51" t="n">
+        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$K$5:$K$22)</f>
+        <v>0</v>
       </c>
       <c r="I6" s="51" t="n">
-        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$K$5:$K$22)</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 2",Revisiones!$I$5:$I$10)</f>
-        <v>0</v>
-      </c>
-      <c r="K6" s="25" t="str">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 2",Revisiones!$H$5:$H$10)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="25" t="str">
         <f aca="false">IF(COUNTIFS(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$A$5:$A$22,"Equipo 2",Flujo!$M$5:$M$22,"?*"))</f>
         <v/>
       </c>
-      <c r="L6" s="24" t="n">
+      <c r="K6" s="24" t="n">
         <f aca="false">SUMIF(Desperdicios!$C$5:$C$44,"Equipo 2",Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="M6" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 2",Revisiones!$H$5:$H$10)</f>
+      <c r="L6" s="51" t="n">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 2",Revisiones!$G$5:$G$10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="51" t="n">
+      <c r="C7" s="51" t="n">
         <f aca="false">COUNTIFS(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$H$5:$H$22,"&gt;=0")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="D7" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$H$5:$H$22)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="24" t="str">
-        <f aca="false">IF(D7&gt;0,E7/D7,"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="24" t="n">
+      <c r="E7" s="24" t="str">
+        <f aca="false">IF(C7&gt;0,D7/C7,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$I$5:$I$22)</f>
         <v>0</v>
       </c>
-      <c r="H7" s="25" t="str">
-        <f aca="false">IF(E7&gt;0,(E7-G7)/E7,"")</f>
-        <v/>
+      <c r="G7" s="25" t="str">
+        <f aca="false">IF(D7&gt;0,(D7-F7)/D7,"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="51" t="n">
+        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$K$5:$K$22)</f>
+        <v>0</v>
       </c>
       <c r="I7" s="51" t="n">
-        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$K$5:$K$22)</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 3",Revisiones!$I$5:$I$10)</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="25" t="str">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 3",Revisiones!$H$5:$H$10)</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="25" t="str">
         <f aca="false">IF(COUNTIFS(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$A$5:$A$22,"Equipo 3",Flujo!$M$5:$M$22,"?*"))</f>
         <v/>
       </c>
-      <c r="L7" s="24" t="n">
+      <c r="K7" s="24" t="n">
         <f aca="false">SUMIF(Desperdicios!$C$5:$C$44,"Equipo 3",Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="M7" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 3",Revisiones!$H$5:$H$10)</f>
+      <c r="L7" s="51" t="n">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 3",Revisiones!$G$5:$G$10)</f>
         <v>0</v>
       </c>
     </row>
@@ -4526,402 +4305,467 @@
         <v>38</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="51" t="n">
+        <v>39</v>
+      </c>
+      <c r="C8" s="51" t="n">
         <f aca="false">COUNTIFS(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$H$5:$H$22,"&gt;=0")</f>
         <v>0</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="D8" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$H$5:$H$22)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="24" t="str">
-        <f aca="false">IF(D8&gt;0,E8/D8,"")</f>
-        <v/>
-      </c>
-      <c r="G8" s="24" t="n">
+      <c r="E8" s="24" t="str">
+        <f aca="false">IF(C8&gt;0,D8/C8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$I$5:$I$22)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="25" t="str">
-        <f aca="false">IF(E8&gt;0,(E8-G8)/E8,"")</f>
-        <v/>
+      <c r="G8" s="25" t="str">
+        <f aca="false">IF(D8&gt;0,(D8-F8)/D8,"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="51" t="n">
+        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$K$5:$K$22)</f>
+        <v>0</v>
       </c>
       <c r="I8" s="51" t="n">
-        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$K$5:$K$22)</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 4",Revisiones!$I$5:$I$10)</f>
-        <v>0</v>
-      </c>
-      <c r="K8" s="25" t="str">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 4",Revisiones!$H$5:$H$10)</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="25" t="str">
         <f aca="false">IF(COUNTIFS(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$A$5:$A$22,"Equipo 4",Flujo!$M$5:$M$22,"?*"))</f>
         <v/>
       </c>
-      <c r="L8" s="24" t="n">
+      <c r="K8" s="24" t="n">
         <f aca="false">SUMIF(Desperdicios!$C$5:$C$44,"Equipo 4",Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="M8" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 4",Revisiones!$H$5:$H$10)</f>
+      <c r="L8" s="51" t="n">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 4",Revisiones!$G$5:$G$10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="51" t="n">
+      <c r="C9" s="51" t="n">
         <f aca="false">COUNTIFS(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$H$5:$H$22,"&gt;=0")</f>
         <v>0</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="D9" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$H$5:$H$22)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="24" t="str">
-        <f aca="false">IF(D9&gt;0,E9/D9,"")</f>
-        <v/>
-      </c>
-      <c r="G9" s="24" t="n">
+      <c r="E9" s="24" t="str">
+        <f aca="false">IF(C9&gt;0,D9/C9,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$I$5:$I$22)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="25" t="str">
-        <f aca="false">IF(E9&gt;0,(E9-G9)/E9,"")</f>
-        <v/>
+      <c r="G9" s="25" t="str">
+        <f aca="false">IF(D9&gt;0,(D9-F9)/D9,"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="51" t="n">
+        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$K$5:$K$22)</f>
+        <v>0</v>
       </c>
       <c r="I9" s="51" t="n">
-        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$K$5:$K$22)</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 5",Revisiones!$I$5:$I$10)</f>
-        <v>0</v>
-      </c>
-      <c r="K9" s="25" t="str">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 5",Revisiones!$H$5:$H$10)</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="25" t="str">
         <f aca="false">IF(COUNTIFS(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$A$5:$A$22,"Equipo 5",Flujo!$M$5:$M$22,"?*"))</f>
         <v/>
       </c>
-      <c r="L9" s="24" t="n">
+      <c r="K9" s="24" t="n">
         <f aca="false">SUMIF(Desperdicios!$C$5:$C$44,"Equipo 5",Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="M9" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 5",Revisiones!$H$5:$H$10)</f>
+      <c r="L9" s="51" t="n">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 5",Revisiones!$G$5:$G$10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D10" s="51" t="n">
+        <v>45</v>
+      </c>
+      <c r="C10" s="51" t="n">
         <f aca="false">COUNTIFS(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$H$5:$H$22,"&gt;=0")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="D10" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$H$5:$H$22)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="24" t="str">
-        <f aca="false">IF(D10&gt;0,E10/D10,"")</f>
-        <v/>
-      </c>
-      <c r="G10" s="24" t="n">
+      <c r="E10" s="24" t="str">
+        <f aca="false">IF(C10&gt;0,D10/C10,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="24" t="n">
         <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$I$5:$I$22)</f>
         <v>0</v>
       </c>
-      <c r="H10" s="25" t="str">
-        <f aca="false">IF(E10&gt;0,(E10-G10)/E10,"")</f>
-        <v/>
+      <c r="G10" s="25" t="str">
+        <f aca="false">IF(D10&gt;0,(D10-F10)/D10,"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="51" t="n">
+        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$K$5:$K$22)</f>
+        <v>0</v>
       </c>
       <c r="I10" s="51" t="n">
-        <f aca="false">SUMIF(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$K$5:$K$22)</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 6",Revisiones!$I$5:$I$10)</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="25" t="str">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 6",Revisiones!$H$5:$H$10)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="25" t="str">
         <f aca="false">IF(COUNTIFS(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$A$5:$A$22,"Equipo 6",Flujo!$M$5:$M$22,"?*"))</f>
         <v/>
       </c>
-      <c r="L10" s="24" t="n">
+      <c r="K10" s="24" t="n">
         <f aca="false">SUMIF(Desperdicios!$C$5:$C$44,"Equipo 6",Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="51" t="n">
-        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 6",Revisiones!$H$5:$H$10)</f>
-        <v>0</v>
+      <c r="L10" s="51" t="n">
+        <f aca="false">SUMIF(Revisiones!$A$5:$A$10,"Equipo 6",Revisiones!$G$5:$G$10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="54"/>
+      <c r="C11" s="55" t="n">
+        <f aca="false">SUM(C5:C10)</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="56" t="n">
+        <f aca="false">SUM(D5:D10)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="56" t="str">
+        <f aca="false">IF(C11&gt;0,D11/C11,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="56" t="n">
+        <f aca="false">SUM(F5:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="57" t="str">
+        <f aca="false">IF(D11&gt;0,(D11-F11)/D11,"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="55" t="n">
+        <f aca="false">SUM(H5:H10)</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="55" t="n">
+        <f aca="false">SUM(I5:I10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="57" t="str">
+        <f aca="false">IF(COUNTIF(Flujo!$M$5:$M$22,"?*")=0,"",COUNTIF(Flujo!$M$5:$M$22,"Sí")/COUNTIF(Flujo!$M$5:$M$22,"?*"))</f>
+        <v/>
+      </c>
+      <c r="K11" s="56" t="n">
+        <f aca="false">SUM(K5:K10)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="55" t="str">
+        <f aca="false">IF(COUNT(Revisiones!$G$5:$G$10)=0,"",AVERAGE(Revisiones!$G$5:$G$10))</f>
+        <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+        <v>132</v>
+      </c>
+      <c r="B14" s="58"/>
+      <c r="C14" s="10" t="s">
+        <v>121</v>
+      </c>
       <c r="D14" s="10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>130</v>
+        <v>63</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>61</v>
+        <v>124</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="K14" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="M14" s="54"/>
+        <v>128</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="55" t="n">
+      <c r="A15" s="59" t="n">
         <v>1</v>
       </c>
+      <c r="C15" s="55" t="n">
+        <f aca="false">COUNTIFS(Flujo!$D$5:$D$22,$A15,Flujo!$H$5:$H$22,"&gt;=0")</f>
+        <v>0</v>
+      </c>
       <c r="D15" s="56" t="n">
-        <f aca="false">SUMIF($C$5:$C$10,$A15,$D$5:$D$10)</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="57" t="n">
-        <f aca="false">SUMIF($C$5:$C$10,$A15,$E$5:$E$10)</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="57" t="str">
-        <f aca="false">IF(D15&gt;0,E15/D15,"")</f>
-        <v/>
-      </c>
-      <c r="G15" s="57" t="n">
-        <f aca="false">SUMIF($C$5:$C$10,$A15,$G$5:$G$10)</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="58" t="str">
-        <f aca="false">IF(E15&gt;0,(E15-G15)/E15,"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="59" t="str">
-        <f aca="false">IF(D15&gt;0,(SUMIF($C$5:$C$10,$A15,$I$5:$I$10)+SUMIF($C$5:$C$10,$A15,$J$5:$J$10))/D15,"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="58" t="str">
-        <f aca="false">IF(COUNTIFS(Flujo!$C$5:$C$22,$A15,Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$C$5:$C$22,$A15,Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$C$5:$C$22,$A15,Flujo!$M$5:$M$22,"?*"))</f>
-        <v/>
-      </c>
-      <c r="K15" s="57" t="n">
+        <f aca="false">SUMIF(Flujo!$D$5:$D$22,$A15,Flujo!$H$5:$H$22)</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="56" t="str">
+        <f aca="false">IF(C15&gt;0,D15/C15,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="56" t="n">
+        <f aca="false">SUMIF(Flujo!$D$5:$D$22,$A15,Flujo!$I$5:$I$22)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="57" t="str">
+        <f aca="false">IF(D15&gt;0,(D15-F15)/D15,"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="60" t="str">
+        <f aca="false">IF(C15&gt;0,SUMIF(Flujo!$D$5:$D$22,$A15,Flujo!$K$5:$K$22)/C15,"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="57" t="str">
+        <f aca="false">IF(COUNTIFS(Flujo!$D$5:$D$22,$A15,Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$D$5:$D$22,$A15,Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$D$5:$D$22,$A15,Flujo!$M$5:$M$22,"?*"))</f>
+        <v/>
+      </c>
+      <c r="J15" s="56" t="n">
         <f aca="false">SUMIF(Desperdicios!$B$5:$B$44,$A15,Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="L15" s="56" t="str">
-        <f aca="false">IF(COUNTIFS(Revisiones!$C$5:$C$10,$A15,Revisiones!$H$5:$H$10,"&gt;=0")=0,"",AVERAGEIFS(Revisiones!$H$5:$H$10,Revisiones!$C$5:$C$10,$A15))</f>
-        <v/>
-      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="55" t="n">
+      <c r="A16" s="59" t="n">
         <v>2</v>
       </c>
+      <c r="C16" s="55" t="n">
+        <f aca="false">COUNTIFS(Flujo!$D$5:$D$22,$A16,Flujo!$H$5:$H$22,"&gt;=0")</f>
+        <v>0</v>
+      </c>
       <c r="D16" s="56" t="n">
-        <f aca="false">SUMIF($C$5:$C$10,$A16,$D$5:$D$10)</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="57" t="n">
-        <f aca="false">SUMIF($C$5:$C$10,$A16,$E$5:$E$10)</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="57" t="str">
-        <f aca="false">IF(D16&gt;0,E16/D16,"")</f>
-        <v/>
-      </c>
-      <c r="G16" s="57" t="n">
-        <f aca="false">SUMIF($C$5:$C$10,$A16,$G$5:$G$10)</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="58" t="str">
-        <f aca="false">IF(E16&gt;0,(E16-G16)/E16,"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="59" t="str">
-        <f aca="false">IF(D16&gt;0,(SUMIF($C$5:$C$10,$A16,$I$5:$I$10)+SUMIF($C$5:$C$10,$A16,$J$5:$J$10))/D16,"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="58" t="str">
-        <f aca="false">IF(COUNTIFS(Flujo!$C$5:$C$22,$A16,Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$C$5:$C$22,$A16,Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$C$5:$C$22,$A16,Flujo!$M$5:$M$22,"?*"))</f>
-        <v/>
-      </c>
-      <c r="K16" s="57" t="n">
+        <f aca="false">SUMIF(Flujo!$D$5:$D$22,$A16,Flujo!$H$5:$H$22)</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="56" t="str">
+        <f aca="false">IF(C16&gt;0,D16/C16,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="56" t="n">
+        <f aca="false">SUMIF(Flujo!$D$5:$D$22,$A16,Flujo!$I$5:$I$22)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="57" t="str">
+        <f aca="false">IF(D16&gt;0,(D16-F16)/D16,"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="60" t="str">
+        <f aca="false">IF(C16&gt;0,SUMIF(Flujo!$D$5:$D$22,$A16,Flujo!$K$5:$K$22)/C16,"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="57" t="str">
+        <f aca="false">IF(COUNTIFS(Flujo!$D$5:$D$22,$A16,Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$D$5:$D$22,$A16,Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$D$5:$D$22,$A16,Flujo!$M$5:$M$22,"?*"))</f>
+        <v/>
+      </c>
+      <c r="J16" s="56" t="n">
         <f aca="false">SUMIF(Desperdicios!$B$5:$B$44,$A16,Desperdicios!$F$5:$F$44)</f>
         <v>0</v>
       </c>
-      <c r="L16" s="56" t="str">
-        <f aca="false">IF(COUNTIFS(Revisiones!$C$5:$C$10,$A16,Revisiones!$H$5:$H$10,"&gt;=0")=0,"",AVERAGEIFS(Revisiones!$H$5:$H$10,Revisiones!$C$5:$C$10,$A16))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="55" t="n">
+        <f aca="false">COUNTIFS(Flujo!$D$5:$D$22,$A17,Flujo!$H$5:$H$22,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="56" t="n">
+        <f aca="false">SUMIF(Flujo!$D$5:$D$22,$A17,Flujo!$H$5:$H$22)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="56" t="str">
+        <f aca="false">IF(C17&gt;0,D17/C17,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="56" t="n">
+        <f aca="false">SUMIF(Flujo!$D$5:$D$22,$A17,Flujo!$I$5:$I$22)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="57" t="str">
+        <f aca="false">IF(D17&gt;0,(D17-F17)/D17,"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="60" t="str">
+        <f aca="false">IF(C17&gt;0,SUMIF(Flujo!$D$5:$D$22,$A17,Flujo!$K$5:$K$22)/C17,"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="57" t="str">
+        <f aca="false">IF(COUNTIFS(Flujo!$D$5:$D$22,$A17,Flujo!$M$5:$M$22,"?*")=0,"",COUNTIFS(Flujo!$D$5:$D$22,$A17,Flujo!$M$5:$M$22,"Sí")/COUNTIFS(Flujo!$D$5:$D$22,$A17,Flujo!$M$5:$M$22,"?*"))</f>
+        <v/>
+      </c>
+      <c r="J17" s="56" t="n">
+        <f aca="false">SUMIF(Desperdicios!$B$5:$B$44,$A17,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="10" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="60" t="s">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="60"/>
-      <c r="C21" s="60"/>
-      <c r="D21" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A21,Desperdicios!$B$5:$B$44,1)</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A21,Desperdicios!$B$5:$B$44,2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="60" t="s">
+      <c r="B22" s="61"/>
+      <c r="C22" s="61"/>
+      <c r="D22" s="24" t="n">
+        <f aca="false">SUMIF(Desperdicios!$D$5:$D$44,$A22,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="51" t="n">
+        <f aca="false">COUNTIF(Desperdicios!$D$5:$D$44,$A22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="60"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A22,Desperdicios!$B$5:$B$44,1)</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A22,Desperdicios!$B$5:$B$44,2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="60" t="s">
+      <c r="B23" s="61"/>
+      <c r="C23" s="61"/>
+      <c r="D23" s="24" t="n">
+        <f aca="false">SUMIF(Desperdicios!$D$5:$D$44,$A23,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="51" t="n">
+        <f aca="false">COUNTIF(Desperdicios!$D$5:$D$44,$A23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="60"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A23,Desperdicios!$B$5:$B$44,1)</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A23,Desperdicios!$B$5:$B$44,2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="60" t="s">
+      <c r="B24" s="61"/>
+      <c r="C24" s="61"/>
+      <c r="D24" s="24" t="n">
+        <f aca="false">SUMIF(Desperdicios!$D$5:$D$44,$A24,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="51" t="n">
+        <f aca="false">COUNTIF(Desperdicios!$D$5:$D$44,$A24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A24,Desperdicios!$B$5:$B$44,1)</f>
-        <v>0</v>
-      </c>
-      <c r="E24" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A24,Desperdicios!$B$5:$B$44,2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="60" t="s">
+      <c r="B25" s="61"/>
+      <c r="C25" s="61"/>
+      <c r="D25" s="24" t="n">
+        <f aca="false">SUMIF(Desperdicios!$D$5:$D$44,$A25,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="51" t="n">
+        <f aca="false">COUNTIF(Desperdicios!$D$5:$D$44,$A25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="61" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="60"/>
-      <c r="C25" s="60"/>
-      <c r="D25" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A25,Desperdicios!$B$5:$B$44,1)</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A25,Desperdicios!$B$5:$B$44,2)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="60" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
+      <c r="B26" s="61"/>
+      <c r="C26" s="61"/>
       <c r="D26" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A26,Desperdicios!$B$5:$B$44,1)</f>
-        <v>0</v>
-      </c>
-      <c r="E26" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A26,Desperdicios!$B$5:$B$44,2)</f>
+        <f aca="false">SUMIF(Desperdicios!$D$5:$D$44,$A26,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="51" t="n">
+        <f aca="false">COUNTIF(Desperdicios!$D$5:$D$44,$A26)</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="60" t="s">
+      <c r="A27" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="61"/>
+      <c r="C27" s="61"/>
+      <c r="D27" s="24" t="n">
+        <f aca="false">SUMIF(Desperdicios!$D$5:$D$44,$A27,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="51" t="n">
+        <f aca="false">COUNTIF(Desperdicios!$D$5:$D$44,$A27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A27,Desperdicios!$B$5:$B$44,1)</f>
-        <v>0</v>
-      </c>
-      <c r="E27" s="24" t="n">
-        <f aca="false">SUMIFS(Desperdicios!$F$5:$F$44,Desperdicios!$D$5:$D$44,$A27,Desperdicios!$B$5:$B$44,2)</f>
+      <c r="B28" s="61"/>
+      <c r="C28" s="61"/>
+      <c r="D28" s="24" t="n">
+        <f aca="false">SUMIF(Desperdicios!$D$5:$D$44,$A28,Desperdicios!$F$5:$F$44)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="51" t="n">
+        <f aca="false">COUNTIF(Desperdicios!$D$5:$D$44,$A28)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A20:C20"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A23:C23"/>
@@ -4929,6 +4773,7 @@
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4937,6 +4782,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>